<commit_message>
Project Kaskan checks in progress
</commit_message>
<xml_diff>
--- a/_ProjectKaskan__Unpublished/Rachael_Robinson_dissertation_file_copies/Brains data for animals/Human Van-Essen & Drury (1997).xlsx
+++ b/_ProjectKaskan__Unpublished/Rachael_Robinson_dissertation_file_copies/Brains data for animals/Human Van-Essen & Drury (1997).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23801"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachael\OneDrive\Documents\PS30094 Dissertation\Brain area data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo-M1-Trait-Data/_ProjectKaskan__Unpublished/Rachael_Robinson_dissertation_file_copies/Brains data for animals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B1F9C3B-8822-4B6F-9D7C-B7C66D894C66}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{1B1F9C3B-8822-4B6F-9D7C-B7C66D894C66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CC7E6E8-AD5C-1546-9F8C-FB9A3973AE1E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4960" yWindow="760" windowWidth="24460" windowHeight="20140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -18,6 +18,19 @@
     <sheet name="Sheet3" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -360,7 +373,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="24">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -916,18 +929,16 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -993,9 +1004,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1033,7 +1044,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1139,7 +1150,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1281,7 +1292,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1290,13 +1301,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E00CC74-2115-41FC-A4FD-BA1982BCA9B4}">
   <dimension ref="A1:S39"/>
-  <sheetFormatPr defaultRowHeight="15.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="8" max="8" width="11.25" customWidth="1"/>
+    <col min="8" max="8" width="11.1640625" customWidth="1"/>
+    <col min="9" max="9" width="8.83203125" customWidth="1"/>
+    <col min="12" max="12" width="8.83203125" customWidth="1"/>
     <col min="19" max="19" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="18.5">
+    <row r="1" spans="1:19" ht="19" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1318,10 +1331,10 @@
       <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="8" t="s">
         <v>34</v>
       </c>
       <c r="J1" t="s">
@@ -1343,7 +1356,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1365,10 +1378,10 @@
       <c r="G2">
         <v>142.673</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="7" t="s">
         <v>35</v>
       </c>
       <c r="J2" t="s">
@@ -1377,23 +1390,21 @@
       <c r="K2" s="4">
         <v>100</v>
       </c>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
       <c r="O2" t="s">
         <v>45</v>
       </c>
-      <c r="P2" s="6">
+      <c r="P2" s="5">
         <f>G2/K2</f>
         <v>1.4267300000000001</v>
       </c>
       <c r="R2" t="s">
         <v>37</v>
       </c>
-      <c r="S2" s="7" t="s">
+      <c r="S2" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="18.5">
+    <row r="3" spans="1:19" ht="19" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1403,27 +1414,27 @@
       <c r="C3" t="s">
         <v>48</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="11" t="s">
+      <c r="I3" s="9" t="s">
         <v>16</v>
       </c>
       <c r="J3" t="s">
         <v>10</v>
       </c>
-      <c r="L3" s="6">
+      <c r="L3" s="5">
         <f t="shared" ref="L3:L37" si="0">B3/$P$3</f>
         <v>3492.898889813081</v>
       </c>
-      <c r="M3" s="6"/>
+      <c r="M3" s="5"/>
       <c r="N3" t="s">
         <v>12</v>
       </c>
       <c r="O3" t="s">
         <v>46</v>
       </c>
-      <c r="P3" s="6">
+      <c r="P3" s="5">
         <f>P2^2</f>
         <v>2.0355584929000003</v>
       </c>
@@ -1434,27 +1445,27 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="18.5">
+    <row r="4" spans="1:19" ht="19" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
         <v>5746</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="I4" s="9" t="s">
         <v>17</v>
       </c>
       <c r="J4" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="5">
         <f t="shared" si="0"/>
         <v>2822.812520515607</v>
       </c>
-      <c r="M4" s="6"/>
+      <c r="M4" s="5"/>
       <c r="N4" t="s">
         <v>12</v>
       </c>
@@ -1465,211 +1476,211 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="18.5">
-      <c r="H5" s="7"/>
-      <c r="I5" s="11" t="s">
+    <row r="5" spans="1:19" ht="19" x14ac:dyDescent="0.2">
+      <c r="H5" s="6"/>
+      <c r="I5" s="9" t="s">
         <v>18</v>
       </c>
       <c r="J5" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M5" s="6"/>
+      <c r="L5" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M5" s="5"/>
       <c r="N5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="18.5">
-      <c r="H6" s="7"/>
-      <c r="I6" s="11" t="s">
+    <row r="6" spans="1:19" ht="19" x14ac:dyDescent="0.2">
+      <c r="H6" s="6"/>
+      <c r="I6" s="9" t="s">
         <v>19</v>
       </c>
       <c r="J6" t="s">
         <v>10</v>
       </c>
-      <c r="L6" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M6" s="6"/>
+      <c r="L6" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M6" s="5"/>
       <c r="N6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="18.5">
-      <c r="H7" s="7"/>
-      <c r="I7" s="11" t="s">
+    <row r="7" spans="1:19" ht="19" x14ac:dyDescent="0.2">
+      <c r="H7" s="6"/>
+      <c r="I7" s="9" t="s">
         <v>20</v>
       </c>
       <c r="J7" t="s">
         <v>10</v>
       </c>
-      <c r="L7" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M7" s="6"/>
+      <c r="L7" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M7" s="5"/>
       <c r="N7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="18.5">
-      <c r="H8" s="7"/>
-      <c r="I8" s="11" t="s">
+    <row r="8" spans="1:19" ht="19" x14ac:dyDescent="0.2">
+      <c r="H8" s="6"/>
+      <c r="I8" s="9" t="s">
         <v>21</v>
       </c>
       <c r="J8" t="s">
         <v>10</v>
       </c>
-      <c r="L8" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M8" s="6"/>
+      <c r="L8" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M8" s="5"/>
       <c r="N8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="18.5">
-      <c r="H9" s="7"/>
-      <c r="I9" s="11" t="s">
+    <row r="9" spans="1:19" ht="19" x14ac:dyDescent="0.2">
+      <c r="H9" s="6"/>
+      <c r="I9" s="9" t="s">
         <v>22</v>
       </c>
       <c r="J9" t="s">
         <v>10</v>
       </c>
-      <c r="L9" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M9" s="6"/>
+      <c r="L9" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M9" s="5"/>
       <c r="N9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="18.5">
-      <c r="H10" s="7"/>
-      <c r="I10" s="11" t="s">
+    <row r="10" spans="1:19" ht="19" x14ac:dyDescent="0.2">
+      <c r="H10" s="6"/>
+      <c r="I10" s="9" t="s">
         <v>23</v>
       </c>
       <c r="J10" t="s">
         <v>10</v>
       </c>
-      <c r="L10" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M10" s="6"/>
+      <c r="L10" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M10" s="5"/>
       <c r="N10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="18.5">
-      <c r="H11" s="7"/>
-      <c r="I11" s="11" t="s">
+    <row r="11" spans="1:19" ht="19" x14ac:dyDescent="0.2">
+      <c r="H11" s="6"/>
+      <c r="I11" s="9" t="s">
         <v>25</v>
       </c>
       <c r="J11" t="s">
         <v>10</v>
       </c>
-      <c r="L11" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M11" s="6"/>
+      <c r="L11" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M11" s="5"/>
       <c r="N11" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="18.5">
-      <c r="H12" s="7"/>
-      <c r="I12" s="11" t="s">
+    <row r="12" spans="1:19" ht="19" x14ac:dyDescent="0.2">
+      <c r="H12" s="6"/>
+      <c r="I12" s="9" t="s">
         <v>26</v>
       </c>
       <c r="J12" t="s">
         <v>10</v>
       </c>
-      <c r="L12" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M12" s="6"/>
+      <c r="L12" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M12" s="5"/>
       <c r="N12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="18.5">
-      <c r="H13" s="7"/>
-      <c r="I13" s="11" t="s">
+    <row r="13" spans="1:19" ht="19" x14ac:dyDescent="0.2">
+      <c r="H13" s="6"/>
+      <c r="I13" s="9" t="s">
         <v>27</v>
       </c>
       <c r="J13" t="s">
         <v>10</v>
       </c>
-      <c r="L13" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M13" s="6"/>
+      <c r="L13" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M13" s="5"/>
       <c r="N13" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="18.5">
-      <c r="H14" s="7"/>
-      <c r="I14" s="11">
+    <row r="14" spans="1:19" ht="19" x14ac:dyDescent="0.2">
+      <c r="H14" s="6"/>
+      <c r="I14" s="9">
         <v>1</v>
       </c>
       <c r="J14" t="s">
         <v>10</v>
       </c>
-      <c r="L14" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M14" s="6"/>
+      <c r="L14" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M14" s="5"/>
       <c r="N14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="18.5">
-      <c r="H15" s="7"/>
-      <c r="I15" s="11">
+    <row r="15" spans="1:19" ht="19" x14ac:dyDescent="0.2">
+      <c r="H15" s="6"/>
+      <c r="I15" s="9">
         <v>2</v>
       </c>
       <c r="J15" t="s">
         <v>10</v>
       </c>
-      <c r="L15" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M15" s="6"/>
+      <c r="L15" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M15" s="5"/>
       <c r="N15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="18.5">
-      <c r="H16" s="7"/>
-      <c r="I16" s="11" t="s">
+    <row r="16" spans="1:19" ht="19" x14ac:dyDescent="0.2">
+      <c r="H16" s="6"/>
+      <c r="I16" s="9" t="s">
         <v>28</v>
       </c>
       <c r="J16" t="s">
         <v>10</v>
       </c>
-      <c r="L16" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M16" s="6"/>
+      <c r="L16" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M16" s="5"/>
       <c r="N16" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="18.5">
+    <row r="17" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>6</v>
       </c>
@@ -1691,339 +1702,339 @@
       <c r="G17">
         <v>0</v>
       </c>
-      <c r="H17" s="7"/>
-      <c r="I17" s="11" t="s">
+      <c r="H17" s="6"/>
+      <c r="I17" s="9" t="s">
         <v>29</v>
       </c>
       <c r="J17" t="s">
         <v>10</v>
       </c>
-      <c r="L17" s="6">
+      <c r="L17" s="5">
         <f t="shared" si="0"/>
         <v>669.10383796419364</v>
       </c>
-      <c r="M17" s="6"/>
+      <c r="M17" s="5"/>
       <c r="N17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="18.5">
-      <c r="H18" s="7"/>
-      <c r="I18" s="11" t="s">
+    <row r="18" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H18" s="6"/>
+      <c r="I18" s="9" t="s">
         <v>30</v>
       </c>
       <c r="J18" t="s">
         <v>10</v>
       </c>
-      <c r="L18" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M18" s="6"/>
+      <c r="L18" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M18" s="5"/>
       <c r="N18" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="18.5">
-      <c r="H19" s="7"/>
-      <c r="I19" s="11" t="s">
+    <row r="19" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H19" s="6"/>
+      <c r="I19" s="9" t="s">
         <v>31</v>
       </c>
       <c r="J19" t="s">
         <v>10</v>
       </c>
-      <c r="L19" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M19" s="6"/>
+      <c r="L19" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M19" s="5"/>
       <c r="N19" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="18.5">
-      <c r="H20" s="7"/>
-      <c r="I20" s="11" t="s">
+    <row r="20" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H20" s="6"/>
+      <c r="I20" s="9" t="s">
         <v>32</v>
       </c>
       <c r="J20" t="s">
         <v>10</v>
       </c>
-      <c r="L20" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M20" s="6"/>
+      <c r="L20" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M20" s="5"/>
       <c r="N20" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="18.5">
-      <c r="H21" s="7"/>
-      <c r="I21" s="11" t="s">
+    <row r="21" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H21" s="6"/>
+      <c r="I21" s="9" t="s">
         <v>33</v>
       </c>
       <c r="J21" t="s">
         <v>10</v>
       </c>
-      <c r="L21" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M21" s="6"/>
+      <c r="L21" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M21" s="5"/>
       <c r="N21" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="18.5">
-      <c r="H22" s="7"/>
-      <c r="I22" s="11"/>
+    <row r="22" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H22" s="6"/>
+      <c r="I22" s="9"/>
       <c r="J22" t="s">
         <v>10</v>
       </c>
-      <c r="L22" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M22" s="6"/>
+      <c r="L22" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M22" s="5"/>
       <c r="N22" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="18.5">
-      <c r="H23" s="7"/>
-      <c r="I23" s="11"/>
+    <row r="23" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H23" s="6"/>
+      <c r="I23" s="9"/>
       <c r="J23" t="s">
         <v>10</v>
       </c>
-      <c r="L23" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M23" s="6"/>
+      <c r="L23" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M23" s="5"/>
       <c r="N23" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="18.5">
-      <c r="H24" s="7"/>
-      <c r="I24" s="11"/>
+    <row r="24" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H24" s="6"/>
+      <c r="I24" s="9"/>
       <c r="J24" t="s">
         <v>10</v>
       </c>
-      <c r="L24" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M24" s="6"/>
+      <c r="L24" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M24" s="5"/>
       <c r="N24" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="18.5">
-      <c r="H25" s="7"/>
-      <c r="I25" s="11"/>
+    <row r="25" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H25" s="6"/>
+      <c r="I25" s="9"/>
       <c r="J25" t="s">
         <v>10</v>
       </c>
-      <c r="L25" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M25" s="6"/>
+      <c r="L25" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M25" s="5"/>
       <c r="N25" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="18.5">
-      <c r="H26" s="7"/>
-      <c r="I26" s="11"/>
+    <row r="26" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H26" s="6"/>
+      <c r="I26" s="9"/>
       <c r="J26" t="s">
         <v>10</v>
       </c>
-      <c r="L26" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M26" s="6"/>
+      <c r="L26" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M26" s="5"/>
       <c r="N26" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="18.5">
-      <c r="H27" s="7"/>
-      <c r="I27" s="11"/>
+    <row r="27" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H27" s="6"/>
+      <c r="I27" s="9"/>
       <c r="J27" t="s">
         <v>10</v>
       </c>
-      <c r="L27" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M27" s="6"/>
+      <c r="L27" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M27" s="5"/>
       <c r="N27" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="18.5">
-      <c r="H28" s="7"/>
-      <c r="I28" s="11"/>
+    <row r="28" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H28" s="6"/>
+      <c r="I28" s="9"/>
       <c r="J28" t="s">
         <v>10</v>
       </c>
-      <c r="L28" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M28" s="6"/>
+      <c r="L28" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M28" s="5"/>
       <c r="N28" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="18.5">
-      <c r="H29" s="7"/>
-      <c r="I29" s="11"/>
+    <row r="29" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H29" s="6"/>
+      <c r="I29" s="9"/>
       <c r="J29" t="s">
         <v>10</v>
       </c>
-      <c r="L29" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M29" s="6"/>
+      <c r="L29" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M29" s="5"/>
       <c r="N29" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="18.5">
-      <c r="H30" s="7"/>
-      <c r="I30" s="11"/>
+    <row r="30" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H30" s="6"/>
+      <c r="I30" s="9"/>
       <c r="J30" t="s">
         <v>10</v>
       </c>
-      <c r="L30" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M30" s="6"/>
+      <c r="L30" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M30" s="5"/>
       <c r="N30" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="18.5">
-      <c r="H31" s="7"/>
-      <c r="I31" s="11"/>
+    <row r="31" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H31" s="6"/>
+      <c r="I31" s="9"/>
       <c r="J31" t="s">
         <v>10</v>
       </c>
-      <c r="L31" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M31" s="6"/>
+      <c r="L31" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M31" s="5"/>
       <c r="N31" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="18.5">
-      <c r="H32" s="7"/>
-      <c r="I32" s="11"/>
+    <row r="32" spans="1:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H32" s="6"/>
+      <c r="I32" s="9"/>
       <c r="J32" t="s">
         <v>10</v>
       </c>
-      <c r="L32" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M32" s="6"/>
+      <c r="L32" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M32" s="5"/>
       <c r="N32" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="8:14" ht="18.5">
-      <c r="H33" s="7"/>
-      <c r="I33" s="11"/>
+    <row r="33" spans="8:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H33" s="6"/>
+      <c r="I33" s="9"/>
       <c r="J33" t="s">
         <v>10</v>
       </c>
-      <c r="L33" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M33" s="6"/>
+      <c r="L33" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M33" s="5"/>
       <c r="N33" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="34" spans="8:14" ht="18.5">
-      <c r="H34" s="7"/>
-      <c r="I34" s="11"/>
+    <row r="34" spans="8:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H34" s="6"/>
+      <c r="I34" s="9"/>
       <c r="J34" t="s">
         <v>10</v>
       </c>
-      <c r="L34" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M34" s="6"/>
+      <c r="L34" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M34" s="5"/>
       <c r="N34" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="8:14" ht="18.5">
-      <c r="H35" s="7"/>
-      <c r="I35" s="11"/>
+    <row r="35" spans="8:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H35" s="6"/>
+      <c r="I35" s="9"/>
       <c r="J35" t="s">
         <v>10</v>
       </c>
-      <c r="L35" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M35" s="6"/>
+      <c r="L35" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M35" s="5"/>
       <c r="N35" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="8:14" ht="18.5">
-      <c r="H36" s="7"/>
-      <c r="I36" s="11"/>
+    <row r="36" spans="8:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H36" s="6"/>
+      <c r="I36" s="9"/>
       <c r="J36" t="s">
         <v>10</v>
       </c>
-      <c r="L36" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M36" s="6"/>
+      <c r="L36" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M36" s="5"/>
       <c r="N36" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="8:14" ht="18.5">
-      <c r="H37" s="7"/>
-      <c r="I37" s="11" t="s">
+    <row r="37" spans="8:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H37" s="6"/>
+      <c r="I37" s="9" t="s">
         <v>24</v>
       </c>
       <c r="J37" t="s">
         <v>10</v>
       </c>
-      <c r="L37" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M37" s="6"/>
+      <c r="L37" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M37" s="5"/>
       <c r="N37" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="8:14">
-      <c r="H38" s="7"/>
-      <c r="I38" s="11"/>
-    </row>
-    <row r="39" spans="8:14">
-      <c r="H39" s="7"/>
-      <c r="I39" s="11"/>
+    <row r="38" spans="8:14" x14ac:dyDescent="0.2">
+      <c r="H38" s="6"/>
+      <c r="I38" s="9"/>
+    </row>
+    <row r="39" spans="8:14" x14ac:dyDescent="0.2">
+      <c r="H39" s="6"/>
+      <c r="I39" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2033,9 +2044,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84A61C2-D7DA-4506-B3EB-B2368D2CDCF7}">
   <dimension ref="A1:S38"/>
-  <sheetFormatPr defaultRowHeight="15.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>1</v>
       </c>
@@ -2076,7 +2087,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2120,11 +2131,11 @@
       <c r="R2" t="s">
         <v>37</v>
       </c>
-      <c r="S2" s="7" t="s">
+      <c r="S2" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:19">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2172,11 +2183,11 @@
       <c r="R3" t="s">
         <v>38</v>
       </c>
-      <c r="S3" s="12" t="s">
+      <c r="S3" s="10" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:19">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2221,7 +2232,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:19">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2257,7 +2268,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:19">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J6" t="s">
         <v>19</v>
       </c>
@@ -2272,7 +2283,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:19">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J7" t="s">
         <v>21</v>
       </c>
@@ -2287,7 +2298,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:19">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>5</v>
       </c>
@@ -2323,7 +2334,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:19">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J9" t="s">
         <v>57</v>
       </c>
@@ -2338,7 +2349,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J10" t="s">
         <v>58</v>
       </c>
@@ -2353,7 +2364,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:19">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J11" t="s">
         <v>59</v>
       </c>
@@ -2368,7 +2379,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:19">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J12" t="s">
         <v>26</v>
       </c>
@@ -2383,7 +2394,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="1:19">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J13" t="s">
         <v>27</v>
       </c>
@@ -2398,7 +2409,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:19">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J14">
         <v>1</v>
       </c>
@@ -2413,7 +2424,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:19">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J15" t="s">
         <v>28</v>
       </c>
@@ -2428,7 +2439,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="1:19">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J16" t="s">
         <v>29</v>
       </c>
@@ -2443,7 +2454,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="10:14">
+    <row r="17" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J17" t="s">
         <v>30</v>
       </c>
@@ -2458,7 +2469,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="10:14">
+    <row r="18" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J18" t="s">
         <v>31</v>
       </c>
@@ -2473,7 +2484,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="10:14">
+    <row r="19" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J19" t="s">
         <v>32</v>
       </c>
@@ -2488,7 +2499,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="10:14">
+    <row r="20" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J20" t="s">
         <v>60</v>
       </c>
@@ -2503,7 +2514,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="21" spans="10:14">
+    <row r="21" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J21" t="s">
         <v>61</v>
       </c>
@@ -2518,7 +2529,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="10:14">
+    <row r="22" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J22" t="s">
         <v>62</v>
       </c>
@@ -2533,41 +2544,41 @@
         <v>54</v>
       </c>
     </row>
-    <row r="36" spans="8:14" ht="18.5">
-      <c r="H36" s="7"/>
-      <c r="I36" s="11"/>
+    <row r="36" spans="8:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H36" s="6"/>
+      <c r="I36" s="9"/>
       <c r="J36" t="s">
         <v>10</v>
       </c>
-      <c r="L36" s="6">
+      <c r="L36" s="5">
         <f t="shared" ref="L36:L37" si="0">B36/$P$3</f>
         <v>0</v>
       </c>
-      <c r="M36" s="6"/>
+      <c r="M36" s="5"/>
       <c r="N36" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="8:14" ht="18.5">
-      <c r="H37" s="7"/>
-      <c r="I37" s="11" t="s">
+    <row r="37" spans="8:14" ht="19" x14ac:dyDescent="0.2">
+      <c r="H37" s="6"/>
+      <c r="I37" s="9" t="s">
         <v>24</v>
       </c>
       <c r="J37" t="s">
         <v>10</v>
       </c>
-      <c r="L37" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M37" s="6"/>
+      <c r="L37" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M37" s="5"/>
       <c r="N37" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="8:14">
-      <c r="H38" s="7"/>
-      <c r="I38" s="11"/>
+    <row r="38" spans="8:14" x14ac:dyDescent="0.2">
+      <c r="H38" s="6"/>
+      <c r="I38" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2578,9 +2589,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{447405E1-856C-4849-B2A9-AEFC7F3F9D53}">
   <dimension ref="A1:S22"/>
-  <sheetFormatPr defaultRowHeight="15.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="13" max="13" width="8.83203125" customWidth="1"/>
+    <col min="18" max="18" width="13.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>1</v>
       </c>
@@ -2621,7 +2636,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2665,11 +2680,11 @@
       <c r="R2" t="s">
         <v>37</v>
       </c>
-      <c r="S2" s="7" t="s">
+      <c r="S2" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:19">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2717,11 +2732,11 @@
       <c r="R3" t="s">
         <v>38</v>
       </c>
-      <c r="S3" s="12" t="s">
+      <c r="S3" s="10" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:19">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="I4" t="s">
         <v>8</v>
       </c>
@@ -2745,7 +2760,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:19">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J5" t="s">
         <v>18</v>
       </c>
@@ -2760,7 +2775,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:19">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J6" t="s">
         <v>19</v>
       </c>
@@ -2775,7 +2790,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:19">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J7" t="s">
         <v>21</v>
       </c>
@@ -2790,7 +2805,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:19">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J8" t="s">
         <v>56</v>
       </c>
@@ -2805,7 +2820,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:19">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J9" t="s">
         <v>57</v>
       </c>
@@ -2820,7 +2835,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>3</v>
       </c>
@@ -2856,7 +2871,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:19">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>4</v>
       </c>
@@ -2892,7 +2907,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:19">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J12" t="s">
         <v>26</v>
       </c>
@@ -2907,7 +2922,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="1:19">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J13" t="s">
         <v>27</v>
       </c>
@@ -2925,7 +2940,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="14" spans="1:19">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J14">
         <v>1</v>
       </c>
@@ -2940,7 +2955,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:19">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J15" t="s">
         <v>28</v>
       </c>
@@ -2955,7 +2970,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="1:19">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J16" t="s">
         <v>29</v>
       </c>
@@ -2970,7 +2985,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="10:14">
+    <row r="17" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J17" t="s">
         <v>30</v>
       </c>
@@ -2985,7 +3000,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="10:14">
+    <row r="18" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J18" t="s">
         <v>31</v>
       </c>
@@ -3000,7 +3015,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="10:14">
+    <row r="19" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J19" t="s">
         <v>32</v>
       </c>
@@ -3015,7 +3030,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="10:14">
+    <row r="20" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J20" t="s">
         <v>60</v>
       </c>
@@ -3030,7 +3045,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="21" spans="10:14">
+    <row r="21" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J21" t="s">
         <v>61</v>
       </c>
@@ -3045,7 +3060,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="10:14">
+    <row r="22" spans="10:14" x14ac:dyDescent="0.2">
       <c r="J22" t="s">
         <v>62</v>
       </c>
@@ -3318,9 +3333,28 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E53ADFD-DE30-4C1C-9625-BDEF53DBAE5E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E53ADFD-DE30-4C1C-9625-BDEF53DBAE5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0D3D4C1-0B7A-4711-8392-9FCAAA9BDF81}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0D3D4C1-0B7A-4711-8392-9FCAAA9BDF81}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>